<commit_message>
Modulo de Inventario V1 - Bodega
</commit_message>
<xml_diff>
--- a/Fase 2/SIGMA_Bitacora_Daily_Scrum.xlsx
+++ b/Fase 2/SIGMA_Bitacora_Daily_Scrum.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\Fase 2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Capstone\SIGMA\Fase 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAB490E-9D52-48E3-9D83-B4F5083D25D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5B09DE9-7D79-48FD-92EE-65037CC4E4D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8272,13 +8272,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="N5:N178" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="N5:N181" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Todo,In Progress,In Review,Done,Blocked"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="P5:P178" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="P5:P181" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Sí,No"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.5"/>
@@ -8415,7 +8413,7 @@
       <c r="K5" s="23"/>
       <c r="L5" s="24">
         <f t="shared" ref="L5:L36" ca="1" si="0">IF($B5="","",IF($J5="Resuelto",IF($K5="","",$K5-$B5),TODAY()-$B5))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -8452,7 +8450,7 @@
       <c r="K6" s="23"/>
       <c r="L6" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -8489,7 +8487,7 @@
       <c r="K7" s="23"/>
       <c r="L7" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -8526,7 +8524,7 @@
       <c r="K8" s="23"/>
       <c r="L8" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.3">
@@ -8563,7 +8561,7 @@
       <c r="K9" s="23"/>
       <c r="L9" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>